<commit_message>
Search matches every word incl. attachment names; sharper injection prompt
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013LaU8KutyVc6GAVj7UGghE
</commit_message>
<xml_diff>
--- a/data/participant_emails.xlsx
+++ b/data/participant_emails.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Email Extraction" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Taxonomy" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email Extraction" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
 </workbook>

</xml_diff>